<commit_message>
Standardize DOCX and XLSX templates on Carbone-style syntax
</commit_message>
<xml_diff>
--- a/corpus/xlsx/level-001/template.xlsx
+++ b/corpus/xlsx/level-001/template.xlsx
@@ -68,38 +68,38 @@
       </c>
       <c r="B1" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">{{title}}</t>
+          <t xml:space="preserve">{d.title}</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">{{customer}}</t>
+          <t xml:space="preserve">{d.customer}</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">{{count}}</t>
+          <t xml:space="preserve">{d.count}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">{{spaced}}</t>
+          <t xml:space="preserve">{d.spaced}</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">{{enabled}}</t>
+          <t xml:space="preserve">{d.enabled}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">{{literal}}</t>
+          <t xml:space="preserve">{d.literal}</t>
         </is>
       </c>
       <c r="B4" s="0">
@@ -109,7 +109,7 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">{{customer}}</t>
+          <t xml:space="preserve">{d.customer}</t>
         </is>
       </c>
     </row>

</xml_diff>